<commit_message>
test: add WenKB manual runtime evidence workflow
</commit_message>
<xml_diff>
--- a/outputs/wenkb-test-book-in-progress/第14小组_基于大模型的个人知识库系统_测试成绩书.xlsx
+++ b/outputs/wenkb-test-book-in-progress/第14小组_基于大模型的个人知识库系统_测试成绩书.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文件封面" sheetId="1" r:id="R8be615ed5725474b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试项目" sheetId="2" r:id="R9d6e0ad9dc0e4f2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI界面" sheetId="3" r:id="Reaf8fc1e7f7b4ffe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行" sheetId="4" r:id="Rd75ea493da1a4dd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="文件封面" sheetId="1" r:id="R4ad4a0728dd34645"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="测试项目" sheetId="2" r:id="R3d94d4b9f5554adc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UI界面" sheetId="3" r:id="R5b5654dcb3fc4be3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="运行" sheetId="4" r:id="Rccbcec2a52a7457f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -20,7 +20,7 @@
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
     <x:numFmt numFmtId="201" formatCode="0%"/>
   </x:numFmts>
-  <x:fonts count="14">
+  <x:fonts count="15">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -98,8 +98,13 @@
       <x:color rgb="FF1F2937"/>
       <x:name val="Microsoft YaHei"/>
     </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF64748B"/>
+      <x:name val="Microsoft YaHei"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="6">
+  <x:fills count="7">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -126,8 +131,13 @@
         <x:fgColor rgb="FFDCE6F1"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="10">
     <x:border>
       <x:left/>
       <x:right/>
@@ -150,11 +160,91 @@
       </x:bottom>
       <x:diagonal/>
     </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:left>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:top>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:top>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:top>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:left>
+      <x:right/>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:right>
+      <x:top/>
+      <x:bottom/>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:left>
+      <x:right/>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right/>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
+    <x:border>
+      <x:left/>
+      <x:right style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:right>
+      <x:top/>
+      <x:bottom style="thin">
+        <x:color rgb="FFA6A6A6"/>
+      </x:bottom>
+      <x:diagonal/>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="54">
+  <x:cellXfs count="83">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -313,11 +403,98 @@
     <x:xf numFmtId="200" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="14" fillId="6" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="9">
+  <x:dxfs count="12">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -414,6 +591,39 @@
       <x:fill>
         <x:patternFill patternType="solid">
           <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF375623"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFE2F0D9"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C0006"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFCE4D6"/>
+        </x:patternFill>
+      </x:fill>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF9C6500"/>
+      </x:font>
+      <x:fill>
+        <x:patternFill patternType="solid">
+          <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
     </x:dxf>
@@ -920,7 +1130,7 @@
     </x:row>
     <x:row r="24" ht="30" customHeight="1">
       <x:c r="A24" s="14" t="str">
-        <x:v>测试项目：核心测试用例；UI界面：页面与流程验收映射；运行：执行汇总、状态判定与缺陷记录。</x:v>
+        <x:v>测试项目：核心测试用例；UI界面：页面与流程验收映射；运行：执行汇总、缺陷记录和实际运行截图留白。</x:v>
       </x:c>
       <x:c r="B24" s="14"/>
       <x:c r="C24" s="14"/>
@@ -3005,7 +3215,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ree0df99a3aac4bfb"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4e3968e754514196"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3281,7 +3491,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra77dc007a26d4627"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbee11af59bef44bc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -3298,6 +3508,7 @@
     <x:col min="6" max="6" width="14" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="24" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
@@ -3311,6 +3522,7 @@
       <x:c r="F1" s="2"/>
       <x:c r="G1" s="2"/>
       <x:c r="H1" s="2"/>
+      <x:c r="I1" s="2"/>
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="2"/>
@@ -3321,6 +3533,7 @@
       <x:c r="F2" s="2"/>
       <x:c r="G2" s="2"/>
       <x:c r="H2" s="2"/>
+      <x:c r="I2" s="2"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="11" t="str">
@@ -3335,6 +3548,7 @@
       <x:c r="F3" s="2"/>
       <x:c r="G3" s="2"/>
       <x:c r="H3" s="2"/>
+      <x:c r="I3" s="2"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="11" t="str">
@@ -3349,6 +3563,7 @@
       <x:c r="F4" s="2"/>
       <x:c r="G4" s="2"/>
       <x:c r="H4" s="2"/>
+      <x:c r="I4" s="2"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="11" t="str">
@@ -3363,6 +3578,7 @@
       <x:c r="F5" s="2"/>
       <x:c r="G5" s="2"/>
       <x:c r="H5" s="2"/>
+      <x:c r="I5" s="2"/>
     </x:row>
     <x:row r="6">
       <x:c r="A6" s="11" t="str">
@@ -3377,6 +3593,7 @@
       <x:c r="F6" s="2"/>
       <x:c r="G6" s="2"/>
       <x:c r="H6" s="2"/>
+      <x:c r="I6" s="2"/>
     </x:row>
     <x:row r="7" ht="38" customHeight="1">
       <x:c r="A7" s="11" t="str">
@@ -3391,6 +3608,7 @@
       <x:c r="F7" s="2"/>
       <x:c r="G7" s="2"/>
       <x:c r="H7" s="2"/>
+      <x:c r="I7" s="2"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="2"/>
@@ -3401,6 +3619,7 @@
       <x:c r="F8" s="2"/>
       <x:c r="G8" s="2"/>
       <x:c r="H8" s="2"/>
+      <x:c r="I8" s="2"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="28" t="str">
@@ -3415,6 +3634,7 @@
       <x:c r="F9" s="2"/>
       <x:c r="G9" s="2"/>
       <x:c r="H9" s="2"/>
+      <x:c r="I9" s="2"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="40" t="str">
@@ -3430,6 +3650,7 @@
       <x:c r="F10" s="2"/>
       <x:c r="G10" s="2"/>
       <x:c r="H10" s="2"/>
+      <x:c r="I10" s="2"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="40" t="str">
@@ -3445,6 +3666,7 @@
       <x:c r="F11" s="2"/>
       <x:c r="G11" s="2"/>
       <x:c r="H11" s="2"/>
+      <x:c r="I11" s="2"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="40" t="str">
@@ -3460,6 +3682,7 @@
       <x:c r="F12" s="2"/>
       <x:c r="G12" s="2"/>
       <x:c r="H12" s="2"/>
+      <x:c r="I12" s="2"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="40" t="str">
@@ -3475,6 +3698,7 @@
       <x:c r="F13" s="2"/>
       <x:c r="G13" s="2"/>
       <x:c r="H13" s="2"/>
+      <x:c r="I13" s="2"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="40" t="str">
@@ -3490,6 +3714,7 @@
       <x:c r="F14" s="2"/>
       <x:c r="G14" s="2"/>
       <x:c r="H14" s="2"/>
+      <x:c r="I14" s="2"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="40" t="str">
@@ -3505,6 +3730,7 @@
       <x:c r="F15" s="2"/>
       <x:c r="G15" s="2"/>
       <x:c r="H15" s="2"/>
+      <x:c r="I15" s="2"/>
     </x:row>
     <x:row r="16">
       <x:c r="A16" s="40" t="str">
@@ -3520,6 +3746,7 @@
       <x:c r="F16" s="2"/>
       <x:c r="G16" s="2"/>
       <x:c r="H16" s="2"/>
+      <x:c r="I16" s="2"/>
     </x:row>
     <x:row r="17">
       <x:c r="A17" s="40" t="str">
@@ -3535,6 +3762,7 @@
       <x:c r="F17" s="2"/>
       <x:c r="G17" s="2"/>
       <x:c r="H17" s="2"/>
+      <x:c r="I17" s="2"/>
     </x:row>
     <x:row r="18">
       <x:c r="A18" s="40" t="str">
@@ -3550,6 +3778,7 @@
       <x:c r="F18" s="2"/>
       <x:c r="G18" s="2"/>
       <x:c r="H18" s="2"/>
+      <x:c r="I18" s="2"/>
     </x:row>
     <x:row r="19">
       <x:c r="A19" s="48" t="str">
@@ -3565,6 +3794,7 @@
       <x:c r="F19" s="2"/>
       <x:c r="G19" s="2"/>
       <x:c r="H19" s="2"/>
+      <x:c r="I19" s="2"/>
     </x:row>
     <x:row r="20">
       <x:c r="A20" s="2"/>
@@ -3575,27 +3805,27 @@
       <x:c r="F20" s="2"/>
       <x:c r="G20" s="2"/>
       <x:c r="H20" s="2"/>
+      <x:c r="I20" s="2"/>
     </x:row>
     <x:row r="21">
       <x:c r="A21" s="25" t="str">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="B21" s="25" t="str">
-        <x:v>每轮测试前填写执行版本、环境和数据基线。</x:v>
-      </x:c>
+        <x:v>执行要求</x:v>
+      </x:c>
+      <x:c r="B21" s="25"/>
       <x:c r="C21" s="25"/>
       <x:c r="D21" s="25"/>
       <x:c r="E21" s="25"/>
       <x:c r="F21" s="25"/>
       <x:c r="G21" s="25"/>
       <x:c r="H21" s="25"/>
+      <x:c r="I21" s="2"/>
     </x:row>
     <x:row r="22" ht="26" customHeight="1">
       <x:c r="A22" s="52" t="str">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B22" s="31" t="str">
-        <x:v>每条用例执行后填写实测结果、确定结果、日期、测试者和证据。</x:v>
+        <x:v>每轮测试前填写执行版本、环境和数据基线。</x:v>
       </x:c>
       <x:c r="C22" s="31"/>
       <x:c r="D22" s="31"/>
@@ -3603,13 +3833,14 @@
       <x:c r="F22" s="31"/>
       <x:c r="G22" s="31"/>
       <x:c r="H22" s="31"/>
+      <x:c r="I22" s="2"/>
     </x:row>
     <x:row r="23" ht="26" customHeight="1">
       <x:c r="A23" s="52" t="str">
-        <x:v>3</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="B23" s="31" t="str">
-        <x:v>失败或阻塞用例必须关联缺陷编号、日志或截图，并在回归后补充结论。</x:v>
+        <x:v>每条用例执行后填写实测结果、确定结果、日期、测试者和证据。</x:v>
       </x:c>
       <x:c r="C23" s="31"/>
       <x:c r="D23" s="31"/>
@@ -3617,13 +3848,14 @@
       <x:c r="F23" s="31"/>
       <x:c r="G23" s="31"/>
       <x:c r="H23" s="31"/>
+      <x:c r="I23" s="2"/>
     </x:row>
     <x:row r="24" ht="26" customHeight="1">
       <x:c r="A24" s="52" t="str">
-        <x:v>4</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B24" s="31" t="str">
-        <x:v>删除与重建测试只使用可恢复测试数据，执行前后保留对象清单。</x:v>
+        <x:v>失败或阻塞用例必须关联缺陷编号、日志或截图，并在回归后补充结论。</x:v>
       </x:c>
       <x:c r="C24" s="31"/>
       <x:c r="D24" s="31"/>
@@ -3631,13 +3863,14 @@
       <x:c r="F24" s="31"/>
       <x:c r="G24" s="31"/>
       <x:c r="H24" s="31"/>
+      <x:c r="I24" s="2"/>
     </x:row>
     <x:row r="25" ht="26" customHeight="1">
       <x:c r="A25" s="52" t="str">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B25" s="31" t="str">
-        <x:v>交付门禁：核心用例全部通过，高优先级缺陷清零或获得明确延期批准。</x:v>
+        <x:v>删除与重建测试只使用可恢复测试数据，执行前后保留对象清单。</x:v>
       </x:c>
       <x:c r="C25" s="31"/>
       <x:c r="D25" s="31"/>
@@ -3645,16 +3878,22 @@
       <x:c r="F25" s="31"/>
       <x:c r="G25" s="31"/>
       <x:c r="H25" s="31"/>
+      <x:c r="I25" s="2"/>
     </x:row>
     <x:row r="26" ht="26" customHeight="1">
-      <x:c r="A26" s="52"/>
-      <x:c r="B26" s="31"/>
+      <x:c r="A26" s="52" t="str">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="B26" s="31" t="str">
+        <x:v>交付门禁：核心用例全部通过，高优先级缺陷清零或获得明确延期批准。</x:v>
+      </x:c>
       <x:c r="C26" s="31"/>
       <x:c r="D26" s="31"/>
       <x:c r="E26" s="31"/>
       <x:c r="F26" s="31"/>
       <x:c r="G26" s="31"/>
       <x:c r="H26" s="31"/>
+      <x:c r="I26" s="2"/>
     </x:row>
     <x:row r="27">
       <x:c r="A27" s="2"/>
@@ -3665,6 +3904,7 @@
       <x:c r="F27" s="2"/>
       <x:c r="G27" s="2"/>
       <x:c r="H27" s="2"/>
+      <x:c r="I27" s="2"/>
     </x:row>
     <x:row r="28">
       <x:c r="A28" s="2"/>
@@ -3675,6 +3915,7 @@
       <x:c r="F28" s="2"/>
       <x:c r="G28" s="2"/>
       <x:c r="H28" s="2"/>
+      <x:c r="I28" s="2"/>
     </x:row>
     <x:row r="29">
       <x:c r="A29" s="28" t="str">
@@ -3699,6 +3940,7 @@
         <x:v>关闭日期</x:v>
       </x:c>
       <x:c r="H29" s="2"/>
+      <x:c r="I29" s="2"/>
     </x:row>
     <x:row r="30" ht="25" customHeight="1">
       <x:c r="A30" s="31" t="str"/>
@@ -3709,6 +3951,7 @@
       <x:c r="F30" s="31" t="str"/>
       <x:c r="G30" s="53"/>
       <x:c r="H30" s="2"/>
+      <x:c r="I30" s="2"/>
     </x:row>
     <x:row r="31" ht="25" customHeight="1">
       <x:c r="A31" s="31" t="str"/>
@@ -3719,6 +3962,7 @@
       <x:c r="F31" s="31" t="str"/>
       <x:c r="G31" s="53"/>
       <x:c r="H31" s="2"/>
+      <x:c r="I31" s="2"/>
     </x:row>
     <x:row r="32" ht="25" customHeight="1">
       <x:c r="A32" s="31" t="str"/>
@@ -3729,6 +3973,7 @@
       <x:c r="F32" s="31" t="str"/>
       <x:c r="G32" s="53"/>
       <x:c r="H32" s="2"/>
+      <x:c r="I32" s="2"/>
     </x:row>
     <x:row r="33" ht="25" customHeight="1">
       <x:c r="A33" s="31" t="str"/>
@@ -3739,6 +3984,7 @@
       <x:c r="F33" s="31" t="str"/>
       <x:c r="G33" s="53"/>
       <x:c r="H33" s="2"/>
+      <x:c r="I33" s="2"/>
     </x:row>
     <x:row r="34" ht="25" customHeight="1">
       <x:c r="A34" s="31" t="str"/>
@@ -3749,16 +3995,984 @@
       <x:c r="F34" s="31" t="str"/>
       <x:c r="G34" s="53"/>
       <x:c r="H34" s="2"/>
+      <x:c r="I34" s="2"/>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="2"/>
+      <x:c r="B35" s="2"/>
+      <x:c r="C35" s="2"/>
+      <x:c r="D35" s="2"/>
+      <x:c r="E35" s="2"/>
+      <x:c r="F35" s="2"/>
+      <x:c r="G35" s="2"/>
+      <x:c r="H35" s="2"/>
+      <x:c r="I35" s="2"/>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="25" t="str">
+        <x:v>项目实际运行情况（待人工执行）</x:v>
+      </x:c>
+      <x:c r="B36" s="25"/>
+      <x:c r="C36" s="25"/>
+      <x:c r="D36" s="25"/>
+      <x:c r="E36" s="25"/>
+      <x:c r="F36" s="25"/>
+      <x:c r="G36" s="25"/>
+      <x:c r="H36" s="25"/>
+      <x:c r="I36" s="25"/>
+    </x:row>
+    <x:row r="37" ht="34" customHeight="1">
+      <x:c r="A37" s="54" t="str">
+        <x:v>依据 docs/test_scorebook_manual_run.md 在隔离副本中手动运行并粘贴截图。本区仅记录运行冒烟证据，不替代 48 条用例执行，也不改变交付判定。</x:v>
+      </x:c>
+      <x:c r="B37" s="54"/>
+      <x:c r="C37" s="54"/>
+      <x:c r="D37" s="54"/>
+      <x:c r="E37" s="54"/>
+      <x:c r="F37" s="54"/>
+      <x:c r="G37" s="54"/>
+      <x:c r="H37" s="54"/>
+      <x:c r="I37" s="54"/>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="2"/>
+      <x:c r="B38" s="2"/>
+      <x:c r="C38" s="2"/>
+      <x:c r="D38" s="2"/>
+      <x:c r="E38" s="2"/>
+      <x:c r="F38" s="2"/>
+      <x:c r="G38" s="2"/>
+      <x:c r="H38" s="2"/>
+      <x:c r="I38" s="2"/>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="56" t="str">
+        <x:v>运行环境记录</x:v>
+      </x:c>
+      <x:c r="B39" s="56"/>
+      <x:c r="C39" s="56"/>
+      <x:c r="D39" s="56"/>
+      <x:c r="E39" s="56"/>
+      <x:c r="F39" s="56"/>
+      <x:c r="G39" s="56"/>
+      <x:c r="H39" s="56"/>
+      <x:c r="I39" s="56"/>
+    </x:row>
+    <x:row r="40" ht="28" customHeight="1">
+      <x:c r="A40" s="59" t="str">
+        <x:v>项目版本</x:v>
+      </x:c>
+      <x:c r="B40" s="41" t="str"/>
+      <x:c r="C40" s="41" t="str"/>
+      <x:c r="D40" s="41" t="str"/>
+      <x:c r="E40" s="59" t="str">
+        <x:v>Git 提交</x:v>
+      </x:c>
+      <x:c r="F40" s="41" t="str"/>
+      <x:c r="G40" s="41" t="str"/>
+      <x:c r="H40" s="59" t="str">
+        <x:v>执行人</x:v>
+      </x:c>
+      <x:c r="I40" s="41" t="str"/>
+    </x:row>
+    <x:row r="41" ht="28" customHeight="1">
+      <x:c r="A41" s="59" t="str">
+        <x:v>操作系统</x:v>
+      </x:c>
+      <x:c r="B41" s="41" t="str"/>
+      <x:c r="C41" s="41" t="str"/>
+      <x:c r="D41" s="41" t="str"/>
+      <x:c r="E41" s="59" t="str">
+        <x:v>浏览器</x:v>
+      </x:c>
+      <x:c r="F41" s="41" t="str"/>
+      <x:c r="G41" s="41" t="str"/>
+      <x:c r="H41" s="59" t="str">
+        <x:v>执行日期</x:v>
+      </x:c>
+      <x:c r="I41" s="60"/>
+    </x:row>
+    <x:row r="42" ht="28" customHeight="1">
+      <x:c r="A42" s="59" t="str">
+        <x:v>后端入口</x:v>
+      </x:c>
+      <x:c r="B42" s="41" t="str">
+        <x:v>http://127.0.0.1:16088/health</x:v>
+      </x:c>
+      <x:c r="C42" s="41" t="str"/>
+      <x:c r="D42" s="41" t="str"/>
+      <x:c r="E42" s="59" t="str">
+        <x:v>前端入口</x:v>
+      </x:c>
+      <x:c r="F42" s="41" t="str">
+        <x:v>http://127.0.0.1:11420</x:v>
+      </x:c>
+      <x:c r="G42" s="41" t="str"/>
+      <x:c r="H42" s="59" t="str">
+        <x:v>数据库</x:v>
+      </x:c>
+      <x:c r="I42" s="41" t="str">
+        <x:v>隔离副本</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="43">
+      <x:c r="A43" s="2"/>
+      <x:c r="B43" s="2"/>
+      <x:c r="C43" s="2"/>
+      <x:c r="D43" s="2"/>
+      <x:c r="E43" s="2"/>
+      <x:c r="F43" s="2"/>
+      <x:c r="G43" s="2"/>
+      <x:c r="H43" s="2"/>
+      <x:c r="I43" s="2"/>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="56" t="str">
+        <x:v>运行证据清单</x:v>
+      </x:c>
+      <x:c r="B44" s="56"/>
+      <x:c r="C44" s="56"/>
+      <x:c r="D44" s="56"/>
+      <x:c r="E44" s="56"/>
+      <x:c r="F44" s="56"/>
+      <x:c r="G44" s="56"/>
+      <x:c r="H44" s="56"/>
+      <x:c r="I44" s="56"/>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="28" t="str">
+        <x:v>编号</x:v>
+      </x:c>
+      <x:c r="B45" s="28" t="str">
+        <x:v>运行场景</x:v>
+      </x:c>
+      <x:c r="C45" s="28"/>
+      <x:c r="D45" s="28" t="str">
+        <x:v>核验要点</x:v>
+      </x:c>
+      <x:c r="E45" s="28"/>
+      <x:c r="F45" s="28" t="str">
+        <x:v>执行结果</x:v>
+      </x:c>
+      <x:c r="G45" s="28" t="str">
+        <x:v>执行日期</x:v>
+      </x:c>
+      <x:c r="H45" s="28" t="str">
+        <x:v>执行者</x:v>
+      </x:c>
+      <x:c r="I45" s="28" t="str">
+        <x:v>截图编号/文件名</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="48" customHeight="1">
+      <x:c r="A46" s="32" t="str">
+        <x:v>S01</x:v>
+      </x:c>
+      <x:c r="B46" s="31" t="str">
+        <x:v>后端启动与健康检查</x:v>
+      </x:c>
+      <x:c r="C46" s="31"/>
+      <x:c r="D46" s="31" t="str">
+        <x:v>本地后端可启动；/health 返回成功且 data.status、data.database 均为 ok。</x:v>
+      </x:c>
+      <x:c r="E46" s="31"/>
+      <x:c r="F46" s="35" t="str">
+        <x:v>待人工执行</x:v>
+      </x:c>
+      <x:c r="G46" s="53"/>
+      <x:c r="H46" s="31" t="str"/>
+      <x:c r="I46" s="31" t="str">
+        <x:v>S01-health.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="48" customHeight="1">
+      <x:c r="A47" s="32" t="str">
+        <x:v>S02</x:v>
+      </x:c>
+      <x:c r="B47" s="31" t="str">
+        <x:v>前端入口与导航</x:v>
+      </x:c>
+      <x:c r="C47" s="31"/>
+      <x:c r="D47" s="31" t="str">
+        <x:v>浏览器工作区可加载，知识库、搜索、聊天和文档集入口可见。</x:v>
+      </x:c>
+      <x:c r="E47" s="31"/>
+      <x:c r="F47" s="35" t="str">
+        <x:v>待人工执行</x:v>
+      </x:c>
+      <x:c r="G47" s="53"/>
+      <x:c r="H47" s="31" t="str"/>
+      <x:c r="I47" s="31" t="str">
+        <x:v>S02-workspace.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="48" customHeight="1">
+      <x:c r="A48" s="32" t="str">
+        <x:v>S03</x:v>
+      </x:c>
+      <x:c r="B48" s="31" t="str">
+        <x:v>模型设置页</x:v>
+      </x:c>
+      <x:c r="C48" s="31"/>
+      <x:c r="D48" s="31" t="str">
+        <x:v>模型设置页可打开；截图不暴露密钥。未配置模型时如实记录。</x:v>
+      </x:c>
+      <x:c r="E48" s="31"/>
+      <x:c r="F48" s="35" t="str">
+        <x:v>待人工执行</x:v>
+      </x:c>
+      <x:c r="G48" s="53"/>
+      <x:c r="H48" s="31" t="str"/>
+      <x:c r="I48" s="31" t="str">
+        <x:v>S03-model-settings.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="48" customHeight="1">
+      <x:c r="A49" s="32" t="str">
+        <x:v>S04</x:v>
+      </x:c>
+      <x:c r="B49" s="31" t="str">
+        <x:v>知识库列表与详情</x:v>
+      </x:c>
+      <x:c r="C49" s="31"/>
+      <x:c r="D49" s="31" t="str">
+        <x:v>知识库页面可用；如创建测试知识库，只在隔离副本中执行。</x:v>
+      </x:c>
+      <x:c r="E49" s="31"/>
+      <x:c r="F49" s="35" t="str">
+        <x:v>待人工执行</x:v>
+      </x:c>
+      <x:c r="G49" s="53"/>
+      <x:c r="H49" s="31" t="str"/>
+      <x:c r="I49" s="31" t="str">
+        <x:v>S04-repository.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="48" customHeight="1">
+      <x:c r="A50" s="32" t="str">
+        <x:v>S05</x:v>
+      </x:c>
+      <x:c r="B50" s="31" t="str">
+        <x:v>测试资料导入与状态</x:v>
+      </x:c>
+      <x:c r="C50" s="31"/>
+      <x:c r="D50" s="31" t="str">
+        <x:v>样例文件上传后可查看数据集和真实索引状态，不将失败或未就绪写成成功。</x:v>
+      </x:c>
+      <x:c r="E50" s="31"/>
+      <x:c r="F50" s="35" t="str">
+        <x:v>待人工执行</x:v>
+      </x:c>
+      <x:c r="G50" s="53"/>
+      <x:c r="H50" s="31" t="str"/>
+      <x:c r="I50" s="31" t="str">
+        <x:v>S05-dataset.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="48" customHeight="1">
+      <x:c r="A51" s="32" t="str">
+        <x:v>S06</x:v>
+      </x:c>
+      <x:c r="B51" s="31" t="str">
+        <x:v>搜索/问答与引用（模型可用时）</x:v>
+      </x:c>
+      <x:c r="C51" s="31"/>
+      <x:c r="D51" s="31" t="str">
+        <x:v>模型和索引可用时核对命中内容及来源；依赖缺失时记录阻塞原因。</x:v>
+      </x:c>
+      <x:c r="E51" s="31"/>
+      <x:c r="F51" s="35" t="str">
+        <x:v>待人工执行</x:v>
+      </x:c>
+      <x:c r="G51" s="53"/>
+      <x:c r="H51" s="31" t="str"/>
+      <x:c r="I51" s="31" t="str">
+        <x:v>S06-search-chat.png</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="2"/>
+      <x:c r="B52" s="2"/>
+      <x:c r="C52" s="2"/>
+      <x:c r="D52" s="2"/>
+      <x:c r="E52" s="2"/>
+      <x:c r="F52" s="2"/>
+      <x:c r="G52" s="2"/>
+      <x:c r="H52" s="2"/>
+      <x:c r="I52" s="2"/>
+    </x:row>
+    <x:row r="53">
+      <x:c r="A53" s="25" t="str">
+        <x:v>运行界面截图（完成对应步骤后粘贴；当前为空白证据位）</x:v>
+      </x:c>
+      <x:c r="B53" s="25"/>
+      <x:c r="C53" s="25"/>
+      <x:c r="D53" s="25"/>
+      <x:c r="E53" s="25"/>
+      <x:c r="F53" s="25"/>
+      <x:c r="G53" s="25"/>
+      <x:c r="H53" s="25"/>
+      <x:c r="I53" s="25"/>
+    </x:row>
+    <x:row r="54">
+      <x:c r="A54" s="63" t="str">
+        <x:v>S01</x:v>
+      </x:c>
+      <x:c r="B54" s="63" t="str">
+        <x:v>后端健康检查响应</x:v>
+      </x:c>
+      <x:c r="C54" s="63"/>
+      <x:c r="D54" s="63"/>
+      <x:c r="E54" s="63"/>
+      <x:c r="F54" s="63"/>
+      <x:c r="G54" s="63"/>
+      <x:c r="H54" s="63"/>
+      <x:c r="I54" s="63"/>
+    </x:row>
+    <x:row r="55" ht="22" customHeight="1">
+      <x:c r="A55" s="74" t="str">
+        <x:v>待粘贴 S01 实际截图</x:v>
+      </x:c>
+      <x:c r="B55" s="75"/>
+      <x:c r="C55" s="75"/>
+      <x:c r="D55" s="75"/>
+      <x:c r="E55" s="75"/>
+      <x:c r="F55" s="75"/>
+      <x:c r="G55" s="75"/>
+      <x:c r="H55" s="75"/>
+      <x:c r="I55" s="76"/>
+    </x:row>
+    <x:row r="56" ht="22" customHeight="1">
+      <x:c r="A56" s="77"/>
+      <x:c r="B56" s="78"/>
+      <x:c r="C56" s="78"/>
+      <x:c r="D56" s="78"/>
+      <x:c r="E56" s="78"/>
+      <x:c r="F56" s="78"/>
+      <x:c r="G56" s="78"/>
+      <x:c r="H56" s="78"/>
+      <x:c r="I56" s="79"/>
+    </x:row>
+    <x:row r="57" ht="22" customHeight="1">
+      <x:c r="A57" s="77"/>
+      <x:c r="B57" s="78"/>
+      <x:c r="C57" s="78"/>
+      <x:c r="D57" s="78"/>
+      <x:c r="E57" s="78"/>
+      <x:c r="F57" s="78"/>
+      <x:c r="G57" s="78"/>
+      <x:c r="H57" s="78"/>
+      <x:c r="I57" s="79"/>
+    </x:row>
+    <x:row r="58" ht="22" customHeight="1">
+      <x:c r="A58" s="77"/>
+      <x:c r="B58" s="78"/>
+      <x:c r="C58" s="78"/>
+      <x:c r="D58" s="78"/>
+      <x:c r="E58" s="78"/>
+      <x:c r="F58" s="78"/>
+      <x:c r="G58" s="78"/>
+      <x:c r="H58" s="78"/>
+      <x:c r="I58" s="79"/>
+    </x:row>
+    <x:row r="59" ht="22" customHeight="1">
+      <x:c r="A59" s="77"/>
+      <x:c r="B59" s="78"/>
+      <x:c r="C59" s="78"/>
+      <x:c r="D59" s="78"/>
+      <x:c r="E59" s="78"/>
+      <x:c r="F59" s="78"/>
+      <x:c r="G59" s="78"/>
+      <x:c r="H59" s="78"/>
+      <x:c r="I59" s="79"/>
+    </x:row>
+    <x:row r="60" ht="22" customHeight="1">
+      <x:c r="A60" s="77"/>
+      <x:c r="B60" s="78"/>
+      <x:c r="C60" s="78"/>
+      <x:c r="D60" s="78"/>
+      <x:c r="E60" s="78"/>
+      <x:c r="F60" s="78"/>
+      <x:c r="G60" s="78"/>
+      <x:c r="H60" s="78"/>
+      <x:c r="I60" s="79"/>
+    </x:row>
+    <x:row r="61" ht="22" customHeight="1">
+      <x:c r="A61" s="80"/>
+      <x:c r="B61" s="81"/>
+      <x:c r="C61" s="81"/>
+      <x:c r="D61" s="81"/>
+      <x:c r="E61" s="81"/>
+      <x:c r="F61" s="81"/>
+      <x:c r="G61" s="81"/>
+      <x:c r="H61" s="81"/>
+      <x:c r="I61" s="82"/>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="2"/>
+      <x:c r="B62" s="2"/>
+      <x:c r="C62" s="2"/>
+      <x:c r="D62" s="2"/>
+      <x:c r="E62" s="2"/>
+      <x:c r="F62" s="2"/>
+      <x:c r="G62" s="2"/>
+      <x:c r="H62" s="2"/>
+      <x:c r="I62" s="2"/>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="63" t="str">
+        <x:v>S02</x:v>
+      </x:c>
+      <x:c r="B63" s="63" t="str">
+        <x:v>WenKB 浏览器工作区与主导航</x:v>
+      </x:c>
+      <x:c r="C63" s="63"/>
+      <x:c r="D63" s="63"/>
+      <x:c r="E63" s="63"/>
+      <x:c r="F63" s="63"/>
+      <x:c r="G63" s="63"/>
+      <x:c r="H63" s="63"/>
+      <x:c r="I63" s="63"/>
+    </x:row>
+    <x:row r="64" ht="22" customHeight="1">
+      <x:c r="A64" s="74" t="str">
+        <x:v>待粘贴 S02 实际截图</x:v>
+      </x:c>
+      <x:c r="B64" s="75"/>
+      <x:c r="C64" s="75"/>
+      <x:c r="D64" s="75"/>
+      <x:c r="E64" s="75"/>
+      <x:c r="F64" s="75"/>
+      <x:c r="G64" s="75"/>
+      <x:c r="H64" s="75"/>
+      <x:c r="I64" s="76"/>
+    </x:row>
+    <x:row r="65" ht="22" customHeight="1">
+      <x:c r="A65" s="77"/>
+      <x:c r="B65" s="78"/>
+      <x:c r="C65" s="78"/>
+      <x:c r="D65" s="78"/>
+      <x:c r="E65" s="78"/>
+      <x:c r="F65" s="78"/>
+      <x:c r="G65" s="78"/>
+      <x:c r="H65" s="78"/>
+      <x:c r="I65" s="79"/>
+    </x:row>
+    <x:row r="66" ht="22" customHeight="1">
+      <x:c r="A66" s="77"/>
+      <x:c r="B66" s="78"/>
+      <x:c r="C66" s="78"/>
+      <x:c r="D66" s="78"/>
+      <x:c r="E66" s="78"/>
+      <x:c r="F66" s="78"/>
+      <x:c r="G66" s="78"/>
+      <x:c r="H66" s="78"/>
+      <x:c r="I66" s="79"/>
+    </x:row>
+    <x:row r="67" ht="22" customHeight="1">
+      <x:c r="A67" s="77"/>
+      <x:c r="B67" s="78"/>
+      <x:c r="C67" s="78"/>
+      <x:c r="D67" s="78"/>
+      <x:c r="E67" s="78"/>
+      <x:c r="F67" s="78"/>
+      <x:c r="G67" s="78"/>
+      <x:c r="H67" s="78"/>
+      <x:c r="I67" s="79"/>
+    </x:row>
+    <x:row r="68" ht="22" customHeight="1">
+      <x:c r="A68" s="77"/>
+      <x:c r="B68" s="78"/>
+      <x:c r="C68" s="78"/>
+      <x:c r="D68" s="78"/>
+      <x:c r="E68" s="78"/>
+      <x:c r="F68" s="78"/>
+      <x:c r="G68" s="78"/>
+      <x:c r="H68" s="78"/>
+      <x:c r="I68" s="79"/>
+    </x:row>
+    <x:row r="69" ht="22" customHeight="1">
+      <x:c r="A69" s="77"/>
+      <x:c r="B69" s="78"/>
+      <x:c r="C69" s="78"/>
+      <x:c r="D69" s="78"/>
+      <x:c r="E69" s="78"/>
+      <x:c r="F69" s="78"/>
+      <x:c r="G69" s="78"/>
+      <x:c r="H69" s="78"/>
+      <x:c r="I69" s="79"/>
+    </x:row>
+    <x:row r="70" ht="22" customHeight="1">
+      <x:c r="A70" s="80"/>
+      <x:c r="B70" s="81"/>
+      <x:c r="C70" s="81"/>
+      <x:c r="D70" s="81"/>
+      <x:c r="E70" s="81"/>
+      <x:c r="F70" s="81"/>
+      <x:c r="G70" s="81"/>
+      <x:c r="H70" s="81"/>
+      <x:c r="I70" s="82"/>
+    </x:row>
+    <x:row r="71">
+      <x:c r="A71" s="2"/>
+      <x:c r="B71" s="2"/>
+      <x:c r="C71" s="2"/>
+      <x:c r="D71" s="2"/>
+      <x:c r="E71" s="2"/>
+      <x:c r="F71" s="2"/>
+      <x:c r="G71" s="2"/>
+      <x:c r="H71" s="2"/>
+      <x:c r="I71" s="2"/>
+    </x:row>
+    <x:row r="72">
+      <x:c r="A72" s="63" t="str">
+        <x:v>S03</x:v>
+      </x:c>
+      <x:c r="B72" s="63" t="str">
+        <x:v>模型设置页面（凭据已脱敏或未配置）</x:v>
+      </x:c>
+      <x:c r="C72" s="63"/>
+      <x:c r="D72" s="63"/>
+      <x:c r="E72" s="63"/>
+      <x:c r="F72" s="63"/>
+      <x:c r="G72" s="63"/>
+      <x:c r="H72" s="63"/>
+      <x:c r="I72" s="63"/>
+    </x:row>
+    <x:row r="73" ht="22" customHeight="1">
+      <x:c r="A73" s="74" t="str">
+        <x:v>待粘贴 S03 实际截图</x:v>
+      </x:c>
+      <x:c r="B73" s="75"/>
+      <x:c r="C73" s="75"/>
+      <x:c r="D73" s="75"/>
+      <x:c r="E73" s="75"/>
+      <x:c r="F73" s="75"/>
+      <x:c r="G73" s="75"/>
+      <x:c r="H73" s="75"/>
+      <x:c r="I73" s="76"/>
+    </x:row>
+    <x:row r="74" ht="22" customHeight="1">
+      <x:c r="A74" s="77"/>
+      <x:c r="B74" s="78"/>
+      <x:c r="C74" s="78"/>
+      <x:c r="D74" s="78"/>
+      <x:c r="E74" s="78"/>
+      <x:c r="F74" s="78"/>
+      <x:c r="G74" s="78"/>
+      <x:c r="H74" s="78"/>
+      <x:c r="I74" s="79"/>
+    </x:row>
+    <x:row r="75" ht="22" customHeight="1">
+      <x:c r="A75" s="77"/>
+      <x:c r="B75" s="78"/>
+      <x:c r="C75" s="78"/>
+      <x:c r="D75" s="78"/>
+      <x:c r="E75" s="78"/>
+      <x:c r="F75" s="78"/>
+      <x:c r="G75" s="78"/>
+      <x:c r="H75" s="78"/>
+      <x:c r="I75" s="79"/>
+    </x:row>
+    <x:row r="76" ht="22" customHeight="1">
+      <x:c r="A76" s="77"/>
+      <x:c r="B76" s="78"/>
+      <x:c r="C76" s="78"/>
+      <x:c r="D76" s="78"/>
+      <x:c r="E76" s="78"/>
+      <x:c r="F76" s="78"/>
+      <x:c r="G76" s="78"/>
+      <x:c r="H76" s="78"/>
+      <x:c r="I76" s="79"/>
+    </x:row>
+    <x:row r="77" ht="22" customHeight="1">
+      <x:c r="A77" s="77"/>
+      <x:c r="B77" s="78"/>
+      <x:c r="C77" s="78"/>
+      <x:c r="D77" s="78"/>
+      <x:c r="E77" s="78"/>
+      <x:c r="F77" s="78"/>
+      <x:c r="G77" s="78"/>
+      <x:c r="H77" s="78"/>
+      <x:c r="I77" s="79"/>
+    </x:row>
+    <x:row r="78" ht="22" customHeight="1">
+      <x:c r="A78" s="77"/>
+      <x:c r="B78" s="78"/>
+      <x:c r="C78" s="78"/>
+      <x:c r="D78" s="78"/>
+      <x:c r="E78" s="78"/>
+      <x:c r="F78" s="78"/>
+      <x:c r="G78" s="78"/>
+      <x:c r="H78" s="78"/>
+      <x:c r="I78" s="79"/>
+    </x:row>
+    <x:row r="79" ht="22" customHeight="1">
+      <x:c r="A79" s="80"/>
+      <x:c r="B79" s="81"/>
+      <x:c r="C79" s="81"/>
+      <x:c r="D79" s="81"/>
+      <x:c r="E79" s="81"/>
+      <x:c r="F79" s="81"/>
+      <x:c r="G79" s="81"/>
+      <x:c r="H79" s="81"/>
+      <x:c r="I79" s="82"/>
+    </x:row>
+    <x:row r="80">
+      <x:c r="A80" s="2"/>
+      <x:c r="B80" s="2"/>
+      <x:c r="C80" s="2"/>
+      <x:c r="D80" s="2"/>
+      <x:c r="E80" s="2"/>
+      <x:c r="F80" s="2"/>
+      <x:c r="G80" s="2"/>
+      <x:c r="H80" s="2"/>
+      <x:c r="I80" s="2"/>
+    </x:row>
+    <x:row r="81">
+      <x:c r="A81" s="63" t="str">
+        <x:v>S04</x:v>
+      </x:c>
+      <x:c r="B81" s="63" t="str">
+        <x:v>隔离测试知识库列表或详情</x:v>
+      </x:c>
+      <x:c r="C81" s="63"/>
+      <x:c r="D81" s="63"/>
+      <x:c r="E81" s="63"/>
+      <x:c r="F81" s="63"/>
+      <x:c r="G81" s="63"/>
+      <x:c r="H81" s="63"/>
+      <x:c r="I81" s="63"/>
+    </x:row>
+    <x:row r="82" ht="22" customHeight="1">
+      <x:c r="A82" s="74" t="str">
+        <x:v>待粘贴 S04 实际截图</x:v>
+      </x:c>
+      <x:c r="B82" s="75"/>
+      <x:c r="C82" s="75"/>
+      <x:c r="D82" s="75"/>
+      <x:c r="E82" s="75"/>
+      <x:c r="F82" s="75"/>
+      <x:c r="G82" s="75"/>
+      <x:c r="H82" s="75"/>
+      <x:c r="I82" s="76"/>
+    </x:row>
+    <x:row r="83" ht="22" customHeight="1">
+      <x:c r="A83" s="77"/>
+      <x:c r="B83" s="78"/>
+      <x:c r="C83" s="78"/>
+      <x:c r="D83" s="78"/>
+      <x:c r="E83" s="78"/>
+      <x:c r="F83" s="78"/>
+      <x:c r="G83" s="78"/>
+      <x:c r="H83" s="78"/>
+      <x:c r="I83" s="79"/>
+    </x:row>
+    <x:row r="84" ht="22" customHeight="1">
+      <x:c r="A84" s="77"/>
+      <x:c r="B84" s="78"/>
+      <x:c r="C84" s="78"/>
+      <x:c r="D84" s="78"/>
+      <x:c r="E84" s="78"/>
+      <x:c r="F84" s="78"/>
+      <x:c r="G84" s="78"/>
+      <x:c r="H84" s="78"/>
+      <x:c r="I84" s="79"/>
+    </x:row>
+    <x:row r="85" ht="22" customHeight="1">
+      <x:c r="A85" s="77"/>
+      <x:c r="B85" s="78"/>
+      <x:c r="C85" s="78"/>
+      <x:c r="D85" s="78"/>
+      <x:c r="E85" s="78"/>
+      <x:c r="F85" s="78"/>
+      <x:c r="G85" s="78"/>
+      <x:c r="H85" s="78"/>
+      <x:c r="I85" s="79"/>
+    </x:row>
+    <x:row r="86" ht="22" customHeight="1">
+      <x:c r="A86" s="77"/>
+      <x:c r="B86" s="78"/>
+      <x:c r="C86" s="78"/>
+      <x:c r="D86" s="78"/>
+      <x:c r="E86" s="78"/>
+      <x:c r="F86" s="78"/>
+      <x:c r="G86" s="78"/>
+      <x:c r="H86" s="78"/>
+      <x:c r="I86" s="79"/>
+    </x:row>
+    <x:row r="87" ht="22" customHeight="1">
+      <x:c r="A87" s="77"/>
+      <x:c r="B87" s="78"/>
+      <x:c r="C87" s="78"/>
+      <x:c r="D87" s="78"/>
+      <x:c r="E87" s="78"/>
+      <x:c r="F87" s="78"/>
+      <x:c r="G87" s="78"/>
+      <x:c r="H87" s="78"/>
+      <x:c r="I87" s="79"/>
+    </x:row>
+    <x:row r="88" ht="22" customHeight="1">
+      <x:c r="A88" s="80"/>
+      <x:c r="B88" s="81"/>
+      <x:c r="C88" s="81"/>
+      <x:c r="D88" s="81"/>
+      <x:c r="E88" s="81"/>
+      <x:c r="F88" s="81"/>
+      <x:c r="G88" s="81"/>
+      <x:c r="H88" s="81"/>
+      <x:c r="I88" s="82"/>
+    </x:row>
+    <x:row r="89">
+      <x:c r="A89" s="2"/>
+      <x:c r="B89" s="2"/>
+      <x:c r="C89" s="2"/>
+      <x:c r="D89" s="2"/>
+      <x:c r="E89" s="2"/>
+      <x:c r="F89" s="2"/>
+      <x:c r="G89" s="2"/>
+      <x:c r="H89" s="2"/>
+      <x:c r="I89" s="2"/>
+    </x:row>
+    <x:row r="90">
+      <x:c r="A90" s="63" t="str">
+        <x:v>S05</x:v>
+      </x:c>
+      <x:c r="B90" s="63" t="str">
+        <x:v>测试资料导入结果与数据集状态</x:v>
+      </x:c>
+      <x:c r="C90" s="63"/>
+      <x:c r="D90" s="63"/>
+      <x:c r="E90" s="63"/>
+      <x:c r="F90" s="63"/>
+      <x:c r="G90" s="63"/>
+      <x:c r="H90" s="63"/>
+      <x:c r="I90" s="63"/>
+    </x:row>
+    <x:row r="91" ht="22" customHeight="1">
+      <x:c r="A91" s="74" t="str">
+        <x:v>待粘贴 S05 实际截图</x:v>
+      </x:c>
+      <x:c r="B91" s="75"/>
+      <x:c r="C91" s="75"/>
+      <x:c r="D91" s="75"/>
+      <x:c r="E91" s="75"/>
+      <x:c r="F91" s="75"/>
+      <x:c r="G91" s="75"/>
+      <x:c r="H91" s="75"/>
+      <x:c r="I91" s="76"/>
+    </x:row>
+    <x:row r="92" ht="22" customHeight="1">
+      <x:c r="A92" s="77"/>
+      <x:c r="B92" s="78"/>
+      <x:c r="C92" s="78"/>
+      <x:c r="D92" s="78"/>
+      <x:c r="E92" s="78"/>
+      <x:c r="F92" s="78"/>
+      <x:c r="G92" s="78"/>
+      <x:c r="H92" s="78"/>
+      <x:c r="I92" s="79"/>
+    </x:row>
+    <x:row r="93" ht="22" customHeight="1">
+      <x:c r="A93" s="77"/>
+      <x:c r="B93" s="78"/>
+      <x:c r="C93" s="78"/>
+      <x:c r="D93" s="78"/>
+      <x:c r="E93" s="78"/>
+      <x:c r="F93" s="78"/>
+      <x:c r="G93" s="78"/>
+      <x:c r="H93" s="78"/>
+      <x:c r="I93" s="79"/>
+    </x:row>
+    <x:row r="94" ht="22" customHeight="1">
+      <x:c r="A94" s="77"/>
+      <x:c r="B94" s="78"/>
+      <x:c r="C94" s="78"/>
+      <x:c r="D94" s="78"/>
+      <x:c r="E94" s="78"/>
+      <x:c r="F94" s="78"/>
+      <x:c r="G94" s="78"/>
+      <x:c r="H94" s="78"/>
+      <x:c r="I94" s="79"/>
+    </x:row>
+    <x:row r="95" ht="22" customHeight="1">
+      <x:c r="A95" s="77"/>
+      <x:c r="B95" s="78"/>
+      <x:c r="C95" s="78"/>
+      <x:c r="D95" s="78"/>
+      <x:c r="E95" s="78"/>
+      <x:c r="F95" s="78"/>
+      <x:c r="G95" s="78"/>
+      <x:c r="H95" s="78"/>
+      <x:c r="I95" s="79"/>
+    </x:row>
+    <x:row r="96" ht="22" customHeight="1">
+      <x:c r="A96" s="77"/>
+      <x:c r="B96" s="78"/>
+      <x:c r="C96" s="78"/>
+      <x:c r="D96" s="78"/>
+      <x:c r="E96" s="78"/>
+      <x:c r="F96" s="78"/>
+      <x:c r="G96" s="78"/>
+      <x:c r="H96" s="78"/>
+      <x:c r="I96" s="79"/>
+    </x:row>
+    <x:row r="97" ht="22" customHeight="1">
+      <x:c r="A97" s="80"/>
+      <x:c r="B97" s="81"/>
+      <x:c r="C97" s="81"/>
+      <x:c r="D97" s="81"/>
+      <x:c r="E97" s="81"/>
+      <x:c r="F97" s="81"/>
+      <x:c r="G97" s="81"/>
+      <x:c r="H97" s="81"/>
+      <x:c r="I97" s="82"/>
+    </x:row>
+    <x:row r="98">
+      <x:c r="A98" s="2"/>
+      <x:c r="B98" s="2"/>
+      <x:c r="C98" s="2"/>
+      <x:c r="D98" s="2"/>
+      <x:c r="E98" s="2"/>
+      <x:c r="F98" s="2"/>
+      <x:c r="G98" s="2"/>
+      <x:c r="H98" s="2"/>
+      <x:c r="I98" s="2"/>
+    </x:row>
+    <x:row r="99">
+      <x:c r="A99" s="63" t="str">
+        <x:v>S06</x:v>
+      </x:c>
+      <x:c r="B99" s="63" t="str">
+        <x:v>搜索/问答结果及引用；模型不可用时改贴阻塞现象</x:v>
+      </x:c>
+      <x:c r="C99" s="63"/>
+      <x:c r="D99" s="63"/>
+      <x:c r="E99" s="63"/>
+      <x:c r="F99" s="63"/>
+      <x:c r="G99" s="63"/>
+      <x:c r="H99" s="63"/>
+      <x:c r="I99" s="63"/>
+    </x:row>
+    <x:row r="100" ht="22" customHeight="1">
+      <x:c r="A100" s="74" t="str">
+        <x:v>待粘贴 S06 实际截图</x:v>
+      </x:c>
+      <x:c r="B100" s="75"/>
+      <x:c r="C100" s="75"/>
+      <x:c r="D100" s="75"/>
+      <x:c r="E100" s="75"/>
+      <x:c r="F100" s="75"/>
+      <x:c r="G100" s="75"/>
+      <x:c r="H100" s="75"/>
+      <x:c r="I100" s="76"/>
+    </x:row>
+    <x:row r="101" ht="22" customHeight="1">
+      <x:c r="A101" s="77"/>
+      <x:c r="B101" s="78"/>
+      <x:c r="C101" s="78"/>
+      <x:c r="D101" s="78"/>
+      <x:c r="E101" s="78"/>
+      <x:c r="F101" s="78"/>
+      <x:c r="G101" s="78"/>
+      <x:c r="H101" s="78"/>
+      <x:c r="I101" s="79"/>
+    </x:row>
+    <x:row r="102" ht="22" customHeight="1">
+      <x:c r="A102" s="77"/>
+      <x:c r="B102" s="78"/>
+      <x:c r="C102" s="78"/>
+      <x:c r="D102" s="78"/>
+      <x:c r="E102" s="78"/>
+      <x:c r="F102" s="78"/>
+      <x:c r="G102" s="78"/>
+      <x:c r="H102" s="78"/>
+      <x:c r="I102" s="79"/>
+    </x:row>
+    <x:row r="103" ht="22" customHeight="1">
+      <x:c r="A103" s="77"/>
+      <x:c r="B103" s="78"/>
+      <x:c r="C103" s="78"/>
+      <x:c r="D103" s="78"/>
+      <x:c r="E103" s="78"/>
+      <x:c r="F103" s="78"/>
+      <x:c r="G103" s="78"/>
+      <x:c r="H103" s="78"/>
+      <x:c r="I103" s="79"/>
+    </x:row>
+    <x:row r="104" ht="22" customHeight="1">
+      <x:c r="A104" s="77"/>
+      <x:c r="B104" s="78"/>
+      <x:c r="C104" s="78"/>
+      <x:c r="D104" s="78"/>
+      <x:c r="E104" s="78"/>
+      <x:c r="F104" s="78"/>
+      <x:c r="G104" s="78"/>
+      <x:c r="H104" s="78"/>
+      <x:c r="I104" s="79"/>
+    </x:row>
+    <x:row r="105" ht="22" customHeight="1">
+      <x:c r="A105" s="77"/>
+      <x:c r="B105" s="78"/>
+      <x:c r="C105" s="78"/>
+      <x:c r="D105" s="78"/>
+      <x:c r="E105" s="78"/>
+      <x:c r="F105" s="78"/>
+      <x:c r="G105" s="78"/>
+      <x:c r="H105" s="78"/>
+      <x:c r="I105" s="79"/>
+    </x:row>
+    <x:row r="106" ht="22" customHeight="1">
+      <x:c r="A106" s="80"/>
+      <x:c r="B106" s="81"/>
+      <x:c r="C106" s="81"/>
+      <x:c r="D106" s="81"/>
+      <x:c r="E106" s="81"/>
+      <x:c r="F106" s="81"/>
+      <x:c r="G106" s="81"/>
+      <x:c r="H106" s="81"/>
+      <x:c r="I106" s="82"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A1:I1"/>
     <x:mergeCell ref="A21:H21"/>
     <x:mergeCell ref="B22:H22"/>
     <x:mergeCell ref="B23:H23"/>
     <x:mergeCell ref="B24:H24"/>
     <x:mergeCell ref="B25:H25"/>
     <x:mergeCell ref="B26:H26"/>
+    <x:mergeCell ref="A36:I36"/>
+    <x:mergeCell ref="A37:I37"/>
+    <x:mergeCell ref="A39:I39"/>
+    <x:mergeCell ref="B40:D40"/>
+    <x:mergeCell ref="F40:G40"/>
+    <x:mergeCell ref="B41:D41"/>
+    <x:mergeCell ref="F41:G41"/>
+    <x:mergeCell ref="B42:D42"/>
+    <x:mergeCell ref="F42:G42"/>
+    <x:mergeCell ref="A44:I44"/>
+    <x:mergeCell ref="B45:C45"/>
+    <x:mergeCell ref="D45:E45"/>
+    <x:mergeCell ref="B46:C46"/>
+    <x:mergeCell ref="D46:E46"/>
+    <x:mergeCell ref="B47:C47"/>
+    <x:mergeCell ref="D47:E47"/>
+    <x:mergeCell ref="B48:C48"/>
+    <x:mergeCell ref="D48:E48"/>
+    <x:mergeCell ref="B49:C49"/>
+    <x:mergeCell ref="D49:E49"/>
+    <x:mergeCell ref="B50:C50"/>
+    <x:mergeCell ref="D50:E50"/>
+    <x:mergeCell ref="B51:C51"/>
+    <x:mergeCell ref="D51:E51"/>
+    <x:mergeCell ref="A53:I53"/>
+    <x:mergeCell ref="B54:I54"/>
+    <x:mergeCell ref="B63:I63"/>
+    <x:mergeCell ref="B72:I72"/>
+    <x:mergeCell ref="B81:I81"/>
+    <x:mergeCell ref="B90:I90"/>
+    <x:mergeCell ref="B99:I99"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="B11:B11">
     <x:cfRule type="cellIs" dxfId="4" priority="1" operator="greaterThan">
@@ -3785,14 +4999,22 @@
       <x:formula>0</x:formula>
     </x:cfRule>
   </x:conditionalFormatting>
-  <x:dataValidations count="1">
+  <x:conditionalFormatting sqref="F46:F51">
+    <x:cfRule type="containsText" dxfId="9" priority="6" operator="containsText" text="通过"/>
+    <x:cfRule type="containsText" dxfId="10" priority="7" operator="containsText" text="失败"/>
+    <x:cfRule type="containsText" dxfId="11" priority="8" operator="containsText" text="阻塞"/>
+  </x:conditionalFormatting>
+  <x:dataValidations count="2">
     <x:dataValidation type="list" sqref="C30:C34">
       <x:formula1>"高,中,低"</x:formula1>
+    </x:dataValidation>
+    <x:dataValidation type="list" sqref="F46:F51">
+      <x:formula1>"待人工执行,通过,失败,阻塞,不适用"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra5f385c3f1fd41e2"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R132dae3e76ab429c"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>